<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-3-17.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-3-17.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-3-17.xlsx
@@ -865,6 +865,9 @@
       <c r="C51" t="str">
         <v>420_松虫草QQ糖_scabiosa white pink_undefined_1bunch</v>
       </c>
+      <c r="F51" t="str">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -923,7 +926,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0610155312914832586335111578040151558153014105106312108510105355351022420</v>
+        <v>0610155312914832586335111578040151558153014105106312108510105355351022425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>